<commit_message>
Lijst met kaders toegevoegd
</commit_message>
<xml_diff>
--- a/LijstKadersZoN-2026.xlsx
+++ b/LijstKadersZoN-2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stichtinggeonovum.sharepoint.com/sites/GI-Beraad-WerkgroepWerkagendaSpoor3/Gedeelde documenten/Werkgroep Werkagenda Spoor 3/LijstKaders/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="210" documentId="8_{D3E9E1F2-F283-49D6-8BB0-E3897529A656}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D9F3AE6C-F182-49BC-BEE6-12287491AC6E}"/>
+  <xr:revisionPtr revIDLastSave="211" documentId="8_{D3E9E1F2-F283-49D6-8BB0-E3897529A656}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9BE087C6-40E0-4B04-9038-41C7DE349164}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{1F434CB9-BE27-46F0-999D-E3FD730707FF}"/>
   </bookViews>
@@ -1473,6 +1473,15 @@
   </cellStyles>
   <dxfs count="14">
     <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -1496,15 +1505,6 @@
         </patternFill>
       </fill>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1748,8 +1748,8 @@
     <tableColumn id="8" xr3:uid="{0176C2D1-A732-4DB6-8D02-766B82808290}" name="Niets doen /  Beinvloeden /  Implementeren &amp; Monitoren / Ontwikkelen &amp; Implementeren / Afmaken &amp; Implementeren / Aanpassen / Schrappen" dataDxfId="4"/>
     <tableColumn id="9" xr3:uid="{54D30F5E-8E74-4C05-B571-1729D70D843A}" name="Niet van het GB, Wel van het GB" dataDxfId="3"/>
     <tableColumn id="10" xr3:uid="{4F33F665-6495-49B5-BDCE-89BCBC13B57C}" name="1e aanspreekpunt / beheerder" dataDxfId="2"/>
-    <tableColumn id="11" xr3:uid="{C75DEF28-5341-4666-8197-E39888C67A75}" name="Korte toelichting" dataDxfId="0"/>
-    <tableColumn id="13" xr3:uid="{306F02C8-B418-4C17-AE73-4298335BFA52}" name="Link" dataDxfId="1"/>
+    <tableColumn id="11" xr3:uid="{C75DEF28-5341-4666-8197-E39888C67A75}" name="Korte toelichting" dataDxfId="1"/>
+    <tableColumn id="13" xr3:uid="{306F02C8-B418-4C17-AE73-4298335BFA52}" name="Link" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6021,7 +6021,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="105" spans="1:12" ht="144" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:12" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A105" s="1" t="s">
         <v>349</v>
       </c>
@@ -6440,6 +6440,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection algorithmName="SHA-512" hashValue="U5t79S5sd70iFOz9/cp8XN22gV6arYtoOTGVVMyWmBebRBNDx4Iz9WgcEmSMb0Nt3Chv6TLa8PGlS5RFb0jxrw==" saltValue="sIMIPaMjhM8+I348MOKLhg==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <hyperlinks>
     <hyperlink ref="A8" r:id="rId1" display="https://digital-strategy.ec.europa.eu/en/library/ethics-guidelines-trustworthy-ai" xr:uid="{E3F3C5E6-C416-4560-BAA6-F35B59425BDE}"/>
     <hyperlink ref="A10" r:id="rId2" display="https://www.digitaleoverheid.nl/overzicht-van-alle-onderwerpen/nieuwe-technologieen-data-en-ethiek/publieke-waarden/" xr:uid="{982B4ED1-47DA-4F3E-8943-C443F09D5A0C}"/>
@@ -6564,15 +6565,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003D9B7C64C3E67D42A30DD965C2A83FD4" ma:contentTypeVersion="12" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="00ee5770985ebe48fb2b685977563e8d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="fc89e4ba-bd28-4971-91f2-1de29b9bd8ef" xmlns:ns3="87bdb72a-2c1e-4cd3-8594-42030c8ccc15" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="df70dbb27f4214d6da5418339ebb67e2" ns2:_="" ns3:_="">
     <xsd:import namespace="fc89e4ba-bd28-4971-91f2-1de29b9bd8ef"/>
@@ -6783,6 +6775,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -6794,14 +6795,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20FF64F0-C653-480D-B706-20C3D8417C5E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E0EB927-F98B-4DB9-9A48-688530AB292D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6820,19 +6813,27 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20FF64F0-C653-480D-B706-20C3D8417C5E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7FA9106C-3C3D-4C08-BCA8-69B795E41314}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="fc89e4ba-bd28-4971-91f2-1de29b9bd8ef"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="fc89e4ba-bd28-4971-91f2-1de29b9bd8ef"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="87bdb72a-2c1e-4cd3-8594-42030c8ccc15"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="87bdb72a-2c1e-4cd3-8594-42030c8ccc15"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>